<commit_message>
STEP 6 FIX (empirical-p, exact-N-match, loo analysis, recurrence core expr source)
</commit_message>
<xml_diff>
--- a/results/CRISPR/crispr_multivariate_results.xlsx
+++ b/results/CRISPR/crispr_multivariate_results.xlsx
@@ -409,16 +409,16 @@
         <v>64</v>
       </c>
       <c r="C2">
-        <v>2.352564796379436</v>
+        <v>2.35256479637944</v>
       </c>
       <c r="D2">
-        <v>0.1668741866827249</v>
+        <v>0.1668741866827244</v>
       </c>
       <c r="E2">
-        <v>0.04919498370509653</v>
+        <v>0.04919498370509637</v>
       </c>
       <c r="F2">
-        <v>0.5773537167338251</v>
+        <v>0.5773537167338262</v>
       </c>
       <c r="G2">
         <v>-0.0004302768203487961</v>
@@ -432,13 +432,13 @@
         <v>64</v>
       </c>
       <c r="C3">
-        <v>0.8754353000483069</v>
+        <v>0.8754353000483078</v>
       </c>
       <c r="D3">
-        <v>0.3131186506050662</v>
+        <v>0.3131186506050659</v>
       </c>
       <c r="E3">
-        <v>-0.01639826553678039</v>
+        <v>-0.01639826553678038</v>
       </c>
       <c r="F3">
         <v>0.7164746897883246</v>
@@ -455,13 +455,13 @@
         <v>64</v>
       </c>
       <c r="C4">
-        <v>0.4521090163395228</v>
+        <v>0.4521090163395231</v>
       </c>
       <c r="D4">
-        <v>0.4419454643407813</v>
+        <v>0.4419454643407812</v>
       </c>
       <c r="E4">
-        <v>0.02372605811668002</v>
+        <v>0.02372605811668001</v>
       </c>
       <c r="F4">
         <v>0.4396710640341311</v>

</xml_diff>

<commit_message>
STEP 7 until 80. (5. Leave-one-HSP90-drug-out robustness analysis)
</commit_message>
<xml_diff>
--- a/results/CRISPR/crispr_multivariate_results.xlsx
+++ b/results/CRISPR/crispr_multivariate_results.xlsx
@@ -409,16 +409,16 @@
         <v>64</v>
       </c>
       <c r="C2">
-        <v>2.35256479637944</v>
+        <v>2.352564796379433</v>
       </c>
       <c r="D2">
-        <v>0.1668741866827244</v>
+        <v>0.1668741866827253</v>
       </c>
       <c r="E2">
-        <v>0.04919498370509637</v>
+        <v>0.04919498370509565</v>
       </c>
       <c r="F2">
-        <v>0.5773537167338262</v>
+        <v>0.5773537167338317</v>
       </c>
       <c r="G2">
         <v>-0.0004302768203487961</v>
@@ -432,16 +432,16 @@
         <v>64</v>
       </c>
       <c r="C3">
-        <v>0.8754353000483078</v>
+        <v>0.8754353000483065</v>
       </c>
       <c r="D3">
-        <v>0.3131186506050659</v>
+        <v>0.3131186506050663</v>
       </c>
       <c r="E3">
-        <v>-0.01639826553678038</v>
+        <v>-0.01639826553678044</v>
       </c>
       <c r="F3">
-        <v>0.7164746897883246</v>
+        <v>0.7164746897883235</v>
       </c>
       <c r="G3">
         <v>-0.00708371020240417</v>
@@ -455,16 +455,16 @@
         <v>64</v>
       </c>
       <c r="C4">
-        <v>0.4521090163395231</v>
+        <v>0.4521090163395224</v>
       </c>
       <c r="D4">
-        <v>0.4419454643407812</v>
+        <v>0.4419454643407817</v>
       </c>
       <c r="E4">
-        <v>0.02372605811668001</v>
+        <v>0.02372605811667993</v>
       </c>
       <c r="F4">
-        <v>0.4396710640341311</v>
+        <v>0.4396710640341325</v>
       </c>
       <c r="G4">
         <v>-0.01752004017163777</v>

</xml_diff>